<commit_message>
Auto: refresh raw URLs for phxnkhlay
</commit_message>
<xml_diff>
--- a/data/phxnkhlay_all_raw.xlsx
+++ b/data/phxnkhlay_all_raw.xlsx
@@ -480,7 +480,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -519,7 +519,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -636,7 +636,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -714,7 +714,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -792,7 +792,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -831,7 +831,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -870,7 +870,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -909,7 +909,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -948,7 +948,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1026,7 +1026,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1065,7 +1065,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1104,7 +1104,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1143,7 +1143,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1260,7 +1260,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1338,7 +1338,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1377,7 +1377,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1416,7 +1416,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1455,7 +1455,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1494,7 +1494,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1572,7 +1572,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1611,7 +1611,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1650,7 +1650,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1728,7 +1728,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1767,7 +1767,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1806,7 +1806,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1845,7 +1845,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1884,7 +1884,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1962,7 +1962,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -2001,7 +2001,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -2040,7 +2040,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -2079,7 +2079,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2118,7 +2118,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -2157,7 +2157,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2196,7 +2196,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -2235,7 +2235,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -2274,7 +2274,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -2313,7 +2313,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -2352,7 +2352,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -2391,7 +2391,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -2430,7 +2430,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -2469,7 +2469,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -2508,7 +2508,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -2547,7 +2547,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -2586,7 +2586,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -2625,7 +2625,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -2664,7 +2664,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -2703,7 +2703,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -2742,7 +2742,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>505640</v>
+        <v>506700</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -2781,7 +2781,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -2859,7 +2859,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -2937,7 +2937,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2976,7 +2976,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -3015,7 +3015,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -3054,7 +3054,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -3093,7 +3093,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -3132,7 +3132,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -3171,7 +3171,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -3210,7 +3210,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -3249,7 +3249,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -3288,7 +3288,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -3327,7 +3327,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -3366,7 +3366,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -3405,7 +3405,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -3444,7 +3444,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -3483,7 +3483,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -3522,7 +3522,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -3561,7 +3561,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -3600,7 +3600,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -3639,7 +3639,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -3678,7 +3678,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -3717,7 +3717,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -3756,7 +3756,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -3795,7 +3795,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -3834,7 +3834,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -3912,7 +3912,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -3951,7 +3951,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>505637</v>
+        <v>506697</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -5160,7 +5160,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -5199,7 +5199,7 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -5238,7 +5238,7 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -5277,7 +5277,7 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -5316,7 +5316,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -5355,7 +5355,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -5394,7 +5394,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -5433,7 +5433,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -5472,7 +5472,7 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -5511,7 +5511,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -5550,7 +5550,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -5589,7 +5589,7 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -5628,7 +5628,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -5667,7 +5667,7 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -5706,7 +5706,7 @@
         </is>
       </c>
       <c r="D136" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -5745,7 +5745,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -5784,7 +5784,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -5823,7 +5823,7 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -5862,7 +5862,7 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -5901,7 +5901,7 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -5940,7 +5940,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -5979,7 +5979,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -6018,7 +6018,7 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -6057,7 +6057,7 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -6096,7 +6096,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -6135,7 +6135,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -6213,7 +6213,7 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -6252,7 +6252,7 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -6291,7 +6291,7 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -6330,7 +6330,7 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>511143</v>
+        <v>506695</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -6369,7 +6369,7 @@
         </is>
       </c>
       <c r="D153" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -6408,7 +6408,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -6447,7 +6447,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -6486,7 +6486,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -6525,7 +6525,7 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -6564,7 +6564,7 @@
         </is>
       </c>
       <c r="D158" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -6603,7 +6603,7 @@
         </is>
       </c>
       <c r="D159" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -6642,7 +6642,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -6681,7 +6681,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -6720,7 +6720,7 @@
         </is>
       </c>
       <c r="D162" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -6759,7 +6759,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -6798,7 +6798,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -6837,7 +6837,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -6876,7 +6876,7 @@
         </is>
       </c>
       <c r="D166" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -6915,7 +6915,7 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -6954,7 +6954,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -6993,7 +6993,7 @@
         </is>
       </c>
       <c r="D169" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -7032,7 +7032,7 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -7071,7 +7071,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -7110,7 +7110,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -7149,7 +7149,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -7188,7 +7188,7 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -7227,7 +7227,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -7266,7 +7266,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -7305,7 +7305,7 @@
         </is>
       </c>
       <c r="D177" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -7344,7 +7344,7 @@
         </is>
       </c>
       <c r="D178" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -7383,7 +7383,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -7422,7 +7422,7 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -7461,7 +7461,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -7500,7 +7500,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -7539,7 +7539,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -7578,7 +7578,7 @@
         </is>
       </c>
       <c r="D184" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -7617,7 +7617,7 @@
         </is>
       </c>
       <c r="D185" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -7656,7 +7656,7 @@
         </is>
       </c>
       <c r="D186" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -7695,7 +7695,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -7734,7 +7734,7 @@
         </is>
       </c>
       <c r="D188" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -7773,7 +7773,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -7812,7 +7812,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -7851,7 +7851,7 @@
         </is>
       </c>
       <c r="D191" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -7890,7 +7890,7 @@
         </is>
       </c>
       <c r="D192" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -7929,7 +7929,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -7968,7 +7968,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -8007,7 +8007,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -8046,7 +8046,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -8085,7 +8085,7 @@
         </is>
       </c>
       <c r="D197" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -8124,7 +8124,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -8163,7 +8163,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -8202,7 +8202,7 @@
         </is>
       </c>
       <c r="D200" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -8241,7 +8241,7 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -8280,7 +8280,7 @@
         </is>
       </c>
       <c r="D202" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -8319,7 +8319,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -8358,7 +8358,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -8397,7 +8397,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -8436,7 +8436,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -8475,7 +8475,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -8514,7 +8514,7 @@
         </is>
       </c>
       <c r="D208" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -8553,7 +8553,7 @@
         </is>
       </c>
       <c r="D209" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -8592,7 +8592,7 @@
         </is>
       </c>
       <c r="D210" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -8631,7 +8631,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -8670,7 +8670,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -8709,7 +8709,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>505636</v>
+        <v>506696</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -8748,7 +8748,7 @@
         </is>
       </c>
       <c r="D214" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -8787,7 +8787,7 @@
         </is>
       </c>
       <c r="D215" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -8826,7 +8826,7 @@
         </is>
       </c>
       <c r="D216" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -8865,7 +8865,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -8904,7 +8904,7 @@
         </is>
       </c>
       <c r="D218" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -8943,7 +8943,7 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -8982,7 +8982,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -9021,7 +9021,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -9060,7 +9060,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -9099,7 +9099,7 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -9138,7 +9138,7 @@
         </is>
       </c>
       <c r="D224" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -9177,7 +9177,7 @@
         </is>
       </c>
       <c r="D225" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -9216,7 +9216,7 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -9255,7 +9255,7 @@
         </is>
       </c>
       <c r="D227" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -9294,7 +9294,7 @@
         </is>
       </c>
       <c r="D228" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -9333,7 +9333,7 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -9372,7 +9372,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -9411,7 +9411,7 @@
         </is>
       </c>
       <c r="D231" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -9450,7 +9450,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -9489,7 +9489,7 @@
         </is>
       </c>
       <c r="D233" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -9528,7 +9528,7 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -9567,7 +9567,7 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -9606,7 +9606,7 @@
         </is>
       </c>
       <c r="D236" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -9645,7 +9645,7 @@
         </is>
       </c>
       <c r="D237" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -9684,7 +9684,7 @@
         </is>
       </c>
       <c r="D238" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -9723,7 +9723,7 @@
         </is>
       </c>
       <c r="D239" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -9762,7 +9762,7 @@
         </is>
       </c>
       <c r="D240" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -9801,7 +9801,7 @@
         </is>
       </c>
       <c r="D241" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -9840,7 +9840,7 @@
         </is>
       </c>
       <c r="D242" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -9879,7 +9879,7 @@
         </is>
       </c>
       <c r="D243" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -9918,7 +9918,7 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>505639</v>
+        <v>506699</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -9957,7 +9957,7 @@
         </is>
       </c>
       <c r="D245" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -9996,7 +9996,7 @@
         </is>
       </c>
       <c r="D246" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -10035,7 +10035,7 @@
         </is>
       </c>
       <c r="D247" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -10074,7 +10074,7 @@
         </is>
       </c>
       <c r="D248" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -10113,7 +10113,7 @@
         </is>
       </c>
       <c r="D249" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -10152,7 +10152,7 @@
         </is>
       </c>
       <c r="D250" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -10191,7 +10191,7 @@
         </is>
       </c>
       <c r="D251" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -10230,7 +10230,7 @@
         </is>
       </c>
       <c r="D252" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -10269,7 +10269,7 @@
         </is>
       </c>
       <c r="D253" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -10308,7 +10308,7 @@
         </is>
       </c>
       <c r="D254" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -10347,7 +10347,7 @@
         </is>
       </c>
       <c r="D255" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -10386,7 +10386,7 @@
         </is>
       </c>
       <c r="D256" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -10425,7 +10425,7 @@
         </is>
       </c>
       <c r="D257" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -10464,7 +10464,7 @@
         </is>
       </c>
       <c r="D258" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -10503,7 +10503,7 @@
         </is>
       </c>
       <c r="D259" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -10542,7 +10542,7 @@
         </is>
       </c>
       <c r="D260" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -10581,7 +10581,7 @@
         </is>
       </c>
       <c r="D261" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -10620,7 +10620,7 @@
         </is>
       </c>
       <c r="D262" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -10659,7 +10659,7 @@
         </is>
       </c>
       <c r="D263" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -10698,7 +10698,7 @@
         </is>
       </c>
       <c r="D264" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -10737,7 +10737,7 @@
         </is>
       </c>
       <c r="D265" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -10776,7 +10776,7 @@
         </is>
       </c>
       <c r="D266" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -10815,7 +10815,7 @@
         </is>
       </c>
       <c r="D267" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -10854,7 +10854,7 @@
         </is>
       </c>
       <c r="D268" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -10893,7 +10893,7 @@
         </is>
       </c>
       <c r="D269" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -10932,7 +10932,7 @@
         </is>
       </c>
       <c r="D270" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -10971,7 +10971,7 @@
         </is>
       </c>
       <c r="D271" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -11010,7 +11010,7 @@
         </is>
       </c>
       <c r="D272" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -11049,7 +11049,7 @@
         </is>
       </c>
       <c r="D273" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -11088,7 +11088,7 @@
         </is>
       </c>
       <c r="D274" t="n">
-        <v>505641</v>
+        <v>506701</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -11127,7 +11127,7 @@
         </is>
       </c>
       <c r="D275" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -11166,7 +11166,7 @@
         </is>
       </c>
       <c r="D276" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -11205,7 +11205,7 @@
         </is>
       </c>
       <c r="D277" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -11244,7 +11244,7 @@
         </is>
       </c>
       <c r="D278" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -11283,7 +11283,7 @@
         </is>
       </c>
       <c r="D279" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -11322,7 +11322,7 @@
         </is>
       </c>
       <c r="D280" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -11361,7 +11361,7 @@
         </is>
       </c>
       <c r="D281" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -11400,7 +11400,7 @@
         </is>
       </c>
       <c r="D282" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -11439,7 +11439,7 @@
         </is>
       </c>
       <c r="D283" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -11478,7 +11478,7 @@
         </is>
       </c>
       <c r="D284" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -11517,7 +11517,7 @@
         </is>
       </c>
       <c r="D285" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -11556,7 +11556,7 @@
         </is>
       </c>
       <c r="D286" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -11595,7 +11595,7 @@
         </is>
       </c>
       <c r="D287" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -11634,7 +11634,7 @@
         </is>
       </c>
       <c r="D288" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -11673,7 +11673,7 @@
         </is>
       </c>
       <c r="D289" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -11712,7 +11712,7 @@
         </is>
       </c>
       <c r="D290" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -11751,7 +11751,7 @@
         </is>
       </c>
       <c r="D291" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -11790,7 +11790,7 @@
         </is>
       </c>
       <c r="D292" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -11829,7 +11829,7 @@
         </is>
       </c>
       <c r="D293" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -11868,7 +11868,7 @@
         </is>
       </c>
       <c r="D294" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -11907,7 +11907,7 @@
         </is>
       </c>
       <c r="D295" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -11946,7 +11946,7 @@
         </is>
       </c>
       <c r="D296" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -11985,7 +11985,7 @@
         </is>
       </c>
       <c r="D297" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -12024,7 +12024,7 @@
         </is>
       </c>
       <c r="D298" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -12063,7 +12063,7 @@
         </is>
       </c>
       <c r="D299" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -12102,7 +12102,7 @@
         </is>
       </c>
       <c r="D300" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -12141,7 +12141,7 @@
         </is>
       </c>
       <c r="D301" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E301" t="inlineStr">
         <is>
@@ -12180,7 +12180,7 @@
         </is>
       </c>
       <c r="D302" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E302" t="inlineStr">
         <is>
@@ -12219,7 +12219,7 @@
         </is>
       </c>
       <c r="D303" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E303" t="inlineStr">
         <is>
@@ -12258,7 +12258,7 @@
         </is>
       </c>
       <c r="D304" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E304" t="inlineStr">
         <is>
@@ -12297,7 +12297,7 @@
         </is>
       </c>
       <c r="D305" t="n">
-        <v>511147</v>
+        <v>506699</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -13506,7 +13506,7 @@
         </is>
       </c>
       <c r="D336" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -13545,7 +13545,7 @@
         </is>
       </c>
       <c r="D337" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -13584,7 +13584,7 @@
         </is>
       </c>
       <c r="D338" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -13623,7 +13623,7 @@
         </is>
       </c>
       <c r="D339" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -13662,7 +13662,7 @@
         </is>
       </c>
       <c r="D340" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -13701,7 +13701,7 @@
         </is>
       </c>
       <c r="D341" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -13740,7 +13740,7 @@
         </is>
       </c>
       <c r="D342" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -13779,7 +13779,7 @@
         </is>
       </c>
       <c r="D343" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -13818,7 +13818,7 @@
         </is>
       </c>
       <c r="D344" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -13857,7 +13857,7 @@
         </is>
       </c>
       <c r="D345" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -13896,7 +13896,7 @@
         </is>
       </c>
       <c r="D346" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -13935,7 +13935,7 @@
         </is>
       </c>
       <c r="D347" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -13974,7 +13974,7 @@
         </is>
       </c>
       <c r="D348" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -14013,7 +14013,7 @@
         </is>
       </c>
       <c r="D349" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -14052,7 +14052,7 @@
         </is>
       </c>
       <c r="D350" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -14091,7 +14091,7 @@
         </is>
       </c>
       <c r="D351" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -14130,7 +14130,7 @@
         </is>
       </c>
       <c r="D352" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -14169,7 +14169,7 @@
         </is>
       </c>
       <c r="D353" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -14208,7 +14208,7 @@
         </is>
       </c>
       <c r="D354" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E354" t="inlineStr">
         <is>
@@ -14247,7 +14247,7 @@
         </is>
       </c>
       <c r="D355" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -14286,7 +14286,7 @@
         </is>
       </c>
       <c r="D356" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E356" t="inlineStr">
         <is>
@@ -14325,7 +14325,7 @@
         </is>
       </c>
       <c r="D357" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -14364,7 +14364,7 @@
         </is>
       </c>
       <c r="D358" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E358" t="inlineStr">
         <is>
@@ -14403,7 +14403,7 @@
         </is>
       </c>
       <c r="D359" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -14442,7 +14442,7 @@
         </is>
       </c>
       <c r="D360" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -14481,7 +14481,7 @@
         </is>
       </c>
       <c r="D361" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -14520,7 +14520,7 @@
         </is>
       </c>
       <c r="D362" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -14559,7 +14559,7 @@
         </is>
       </c>
       <c r="D363" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E363" t="inlineStr">
         <is>
@@ -14598,7 +14598,7 @@
         </is>
       </c>
       <c r="D364" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -14637,7 +14637,7 @@
         </is>
       </c>
       <c r="D365" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E365" t="inlineStr">
         <is>
@@ -14676,7 +14676,7 @@
         </is>
       </c>
       <c r="D366" t="n">
-        <v>511148</v>
+        <v>506700</v>
       </c>
       <c r="E366" t="inlineStr">
         <is>

</xml_diff>